<commit_message>
pushing back FYIbFP to 2026
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/FYIbFP/First Year Impacted by Future Policies.xlsx
+++ b/InputData/ctrl-settings/FYIbFP/First Year Impacted by Future Policies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\ctrl-settings\FYIBFP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\ctrl-settings\FYIbFP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40B39A16-7942-445D-B9FD-81B8504A3857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E6FA6DE-B671-4527-B218-84831E0DC5C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5460" yWindow="1920" windowWidth="21600" windowHeight="12525" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -411,59 +411,59 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -480,19 +480,19 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>